<commit_message>
data(kashmir): refresh route codes — off-network rural codes district-corrected
Sync engine dac9396: route codes for rural off-network terminals now carry the
correct district and distinct ids (Kangan/Manigam -> GB & distinct, Pampore -> PW,
Safapora -> GB). Letter suffixes 8 -> 6 (the remaining are legitimate same-terminal
"5A/5B" pairs). routes.json / log.json / CSV / geojson + RTO & pretty workbooks
regenerated; 615 codes embedded, 0 TMP, 0 dashes, 0 duplicates. Plan unchanged:
172 routes / 1,005 buses / 30 SSCL trunks.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/route-rationalization-kashmir/Kashmir_Route_Frequency_Plan_v3.3.9_RTO.xlsx
+++ b/public/route-rationalization-kashmir/Kashmir_Route_Frequency_Plan_v3.3.9_RTO.xlsx
@@ -12299,7 +12299,7 @@
     <row r="101">
       <c r="A101" s="35" t="inlineStr">
         <is>
-          <t>SRSR10102507</t>
+          <t>SRGB10952551</t>
         </is>
       </c>
       <c r="B101" s="35" t="inlineStr">
@@ -30031,7 +30031,7 @@
     <row r="263">
       <c r="A263" s="41" t="inlineStr">
         <is>
-          <t>SRSR10102507</t>
+          <t>SRGB10952551</t>
         </is>
       </c>
       <c r="B263" s="41" t="inlineStr">
@@ -39805,7 +39805,7 @@
     <row r="352">
       <c r="A352" s="41" t="inlineStr">
         <is>
-          <t>SRSR10102507</t>
+          <t>SRGB10952551</t>
         </is>
       </c>
       <c r="B352" s="41" t="inlineStr">
@@ -67675,7 +67675,7 @@
     <row r="609">
       <c r="A609" s="60" t="inlineStr">
         <is>
-          <t>SRBG10020907</t>
+          <t>SRBG10720948</t>
         </is>
       </c>
       <c r="B609" s="60" t="inlineStr">
@@ -67993,7 +67993,7 @@
     <row r="612">
       <c r="A612" s="66" t="inlineStr">
         <is>
-          <t>SRSR10100955A</t>
+          <t>SRGB10420992</t>
         </is>
       </c>
       <c r="B612" s="66" t="inlineStr">
@@ -68099,7 +68099,7 @@
     <row r="613">
       <c r="A613" s="66" t="inlineStr">
         <is>
-          <t>SRSR10100955B</t>
+          <t>SRGB10380919</t>
         </is>
       </c>
       <c r="B613" s="66" t="inlineStr">

</xml_diff>